<commit_message>
fix(carga-solta): reimportação preserva CE, Cliente e Viagem (etapa 1, M01)
Migration 173 redefine import_breakbulk_manifest_transactional: B/L
existente recebe só o que o arquivo traz; o CE nunca é gravado pelo
Manifesto BB nem pelo B/L avulso (coluna CE ignorada com aviso); CNPJ de
outro Cliente só troca com aceite pelo relink_bl_customer; rota de B/L
faturado pede confirmação de faturamento; B/L em COD mantém o POD; POD
corrigido desvincula o Manifesto Mercante; B/L de outra Viagem recusa o
lote; sugestão por nome gravada; rastro no Histórico (ADR 0078, itens 1
e 14).

A prévia dos três pontos de entrada confere os B/Ls já gravados e o
resultado lista novos, corrigidos, sem mudança e pendências. Modelos de
planilha sem a coluna CE. Os 6 it.fails de auditoriaImportacaoCargaSolta
viraram it, com 5 checagens novas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AFbzisLbhwnd9hRweKXeZ2
</commit_message>
<xml_diff>
--- a/public/templates/carga-solta-modelo.xlsx
+++ b/public/templates/carga-solta-modelo.xlsx
@@ -397,46 +397,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:L4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>BL</v>
       </c>
       <c r="B1" t="str">
-        <v>CE</v>
+        <v>MAQUINAS</v>
       </c>
       <c r="C1" t="str">
-        <v>MAQUINAS</v>
+        <v>PACKAGES</v>
       </c>
       <c r="D1" t="str">
-        <v>PACKAGES</v>
+        <v>PACKAGES TOTAL</v>
       </c>
       <c r="E1" t="str">
-        <v>PACKAGES TOTAL</v>
+        <v>WEIGHT (TON)</v>
       </c>
       <c r="F1" t="str">
-        <v>WEIGHT (TON)</v>
+        <v>CBM (M3)</v>
       </c>
       <c r="G1" t="str">
-        <v>CBM (M3)</v>
+        <v>SHIPPER</v>
       </c>
       <c r="H1" t="str">
-        <v>SHIPPER</v>
+        <v>CONSIGNEE</v>
       </c>
       <c r="I1" t="str">
-        <v>CONSIGNEE</v>
+        <v>NOTIFY</v>
       </c>
       <c r="J1" t="str">
-        <v>NOTIFY</v>
+        <v>CNPJ</v>
       </c>
       <c r="K1" t="str">
-        <v>CNPJ</v>
+        <v>POL</v>
       </c>
       <c r="L1" t="str">
-        <v>POL</v>
-      </c>
-      <c r="M1" t="str">
         <v>POD</v>
       </c>
     </row>
@@ -445,39 +442,36 @@
         <v>CCSV22ZJGVIT001A</v>
       </c>
       <c r="B2" t="str">
-        <v>122605051526081</v>
+        <v>8</v>
       </c>
       <c r="C2" t="str">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="D2" t="str">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E2" t="str">
-        <v>32</v>
+        <v>259,312</v>
       </c>
       <c r="F2" t="str">
-        <v>259,312</v>
+        <v>1217,109</v>
       </c>
       <c r="G2" t="str">
-        <v>1217,109</v>
+        <v>SANY INTERNATIONAL (HONG KONG)</v>
       </c>
       <c r="H2" t="str">
-        <v>SANY INTERNATIONAL (HONG KONG)</v>
+        <v>TIMBRO TRADING S.A</v>
       </c>
       <c r="I2" t="str">
-        <v>TIMBRO TRADING S.A</v>
+        <v>SANY IMPORTACAO E EXPORTACAO</v>
       </c>
       <c r="J2" t="str">
-        <v>SANY IMPORTACAO E EXPORTACAO</v>
+        <v>12345678000195</v>
       </c>
       <c r="K2" t="str">
-        <v>12345678000195</v>
+        <v>CNNSA</v>
       </c>
       <c r="L2" t="str">
-        <v>CNNSA</v>
-      </c>
-      <c r="M2" t="str">
         <v>BRVIT</v>
       </c>
     </row>
@@ -486,39 +480,36 @@
         <v>CCSV22ZJGVIT002A</v>
       </c>
       <c r="B3" t="str">
-        <v>122605051527991</v>
+        <v>10</v>
       </c>
       <c r="C3" t="str">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D3" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E3" t="str">
-        <v>30</v>
+        <v>135,263</v>
       </c>
       <c r="F3" t="str">
-        <v>135,263</v>
+        <v>564,803</v>
       </c>
       <c r="G3" t="str">
-        <v>564,803</v>
+        <v>SANY SOUTH EAST ASIA PTE</v>
       </c>
       <c r="H3" t="str">
-        <v>SANY SOUTH EAST ASIA PTE</v>
+        <v>TIMBRO TRADING S.A</v>
       </c>
       <c r="I3" t="str">
-        <v>TIMBRO TRADING S.A</v>
+        <v>SANY IMPORTACAO E EXPORTACAO</v>
       </c>
       <c r="J3" t="str">
-        <v>SANY IMPORTACAO E EXPORTACAO</v>
+        <v>12345678000195</v>
       </c>
       <c r="K3" t="str">
-        <v>12345678000195</v>
+        <v>CNQDG</v>
       </c>
       <c r="L3" t="str">
-        <v>CNQDG</v>
-      </c>
-      <c r="M3" t="str">
         <v>BRVIT</v>
       </c>
     </row>
@@ -527,45 +518,42 @@
         <v>CCSV22ZJGVIT003A</v>
       </c>
       <c r="B4" t="str">
-        <v>122605051528106</v>
+        <v>8</v>
       </c>
       <c r="C4" t="str">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D4" t="str">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E4" t="str">
-        <v>24</v>
+        <v>177,120</v>
       </c>
       <c r="F4" t="str">
-        <v>177,120</v>
+        <v>810,106</v>
       </c>
       <c r="G4" t="str">
-        <v>810,106</v>
+        <v>SANY SOUTH EAST ASIA PTE</v>
       </c>
       <c r="H4" t="str">
-        <v>SANY SOUTH EAST ASIA PTE</v>
+        <v>TIMBRO TRADING S.A</v>
       </c>
       <c r="I4" t="str">
-        <v>TIMBRO TRADING S.A</v>
+        <v>SANY IMPORTACAO E EXPORTACAO</v>
       </c>
       <c r="J4" t="str">
-        <v>SANY IMPORTACAO E EXPORTACAO</v>
+        <v>12345678000195</v>
       </c>
       <c r="K4" t="str">
-        <v>12345678000195</v>
+        <v>CNQDG</v>
       </c>
       <c r="L4" t="str">
-        <v>CNQDG</v>
-      </c>
-      <c r="M4" t="str">
         <v>BRSSA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>